<commit_message>
Add Amazon JP search ASINs to Sheet2 column G
Parses the JP search queries in column D (excluding brand terms) and stores the union of first-page Amazon.co.jp search result ASINs in column G for the 12 highlighted ad groups.
</commit_message>
<xml_diff>
--- a/work_filled.xlsx
+++ b/work_filled.xlsx
@@ -7888,7 +7888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="97.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7927,6 +7927,11 @@
           <t>추가 사유</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Amazon JP 검색(1페이지) ASIN 합산</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="17.25" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -7960,6 +7965,11 @@
           <t>소형견/ミニ 라인; 스킨/소화/체중/알러지 케어 키워드 유사</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>B09M84SDFN,B0D3FXM3S4,B08SC7PZLV,B07S9XMY44,B08TBFLM8K,B0BY94F25X,B07PKM49Z1,B0D1XQFV1F,B0DX5GPS7Z,B09SPT31SV,B0GCLLSXVJ,B0BY95FH6K,B0G19NPB5T,B077Q5K4YB,B087F88LJS,B0GCMK97CG,B0C27L7X7D,B0B57WG2HT,B0C27KV5X3,B0GCMD6XTF,B0GCLLY8K4,B0GCMZ5V17,B07X1WQWYZ,B08T8C92TG,B00A8O8PA0,B07Y1S4RMV,B0DK8RQFVS,B075MZLM1K,B075MZN12T,B0G56KGPRV,B01N75JV14,B0FVDT8R1F,B0DWMJ53Z3,B09G652JK9,B00DLTBV4Q,B0FVL5YR5L,B0F3JYKFHG,B0873C3VNJ,B0FVFDFZXG,B0BHHLNYXV,B07QGX3K32,B0DK8S2F7X,B0DZX9778S,B0FJG3FYB6,B0FVDNG4G1,B0DJVDQWDW,B0D3GSR736,B0DQ7ZK222,B08NP6ZHTJ,B08NVT445G,B08NPRG7WF,B0DQ8231CK,B0DQ7YVV4Q,B0DKF7QPS6,B0CPY165M5,B0BHHL9M6B,B08M5F8XD7,B08NP9ZZZ1,B0DK8RHYX6,B0DQ7XFHCZ,B087LR5GY3,B0DN1P332G,B0DN1H8D78,B0DN1Q8S52,B0DN1JTP5L,B0DN1H4BHN,B0DN1KJQQD,B0DN1LDLG9,B0DN1PM7KH,B0DN1PK6XK,B0DN1K5Q55,B0DSZWN97N,B0DN1KCZ43,B00DU5681W,B0DK8Q7RCB,B0CJHQMSMQ,B09T33GCR3,B06XBKZKSY,B0BY954JJR,B0CJHM5WNP,B01N47EL7T,B0BY92VNKW,B0BY9647B1,B0BY971391,B06XBWFSQ7,B00ZHE5XNS,B0CZXN6YD2,B0BXCN1MYL,B0DKNF6GRK,B0F2FCC3ZG,B06XC1WH9C,B085956C14,B0B5743XTQ,B0GCMD8KVZ,B0FNN2MGCT,B09T9PR8P8,B0BZCBB7FS,B09CL2G3YR,B0B8CNCTKV,B07VC6Z5YZ,B00UGN90NY,B0BLGSGRSX,B06XFTN1VK,B0FKGK87YS,B081MPJM31,B07GXJCW4V,B086GNFX5N,B01J4U1T5G,B00EN6QSIU,B014R2804O,B014QS48GI,B0DLWWGTQV,B00UGN9CK0,B07B2TC59J,B0812FZSW2,B097P5BXJ6</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="17.25" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -7993,6 +8003,11 @@
           <t>초소형견/미니XS 키워드 일치; 위장/피부 케어 성격 유사</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>B09T9PR8P8,B07WHC9BBH,B001GFW718,B0BWJ3HYVX,B08DNNPMGB,B0FLW77YHY,B09XTFMZPP,B07FSF17J9,B0DB5R74LQ,B001GFS9BA,B00569WY5Y,B07V5GB8PB,B005IITVTU,B07B4F31JG,B00EN6QSIU,B081MPJM31,B0D1Y8GYSG,B09WFYKW7P,B01J4U1MUS,B00F5P2XUK,B01CC8SEXM,B0CJ4Y6SHM,B0DBQ5TCVM,B0CQ2NQZPM,B01CC8SAM2,B08DNNPMFV,B0D1XWLYTW,B01CC8SF1S,B00EN6QPTM,B01CC8SEZA,B09F8W8RVM,B09T8YHF9F,B0D1Y42HMH,B007M68BFQ,B01CC8SF54,B08KSZS66X,B01CC8SAQS,B0CJ4VGG2H,B00F5P7GO8,B007M68BFG,B00F5OM1RG,B0CZKV8P71,B00EN6QN9Y,B01D2VRRVI,B0B8YWV3DT,B00F5PC0RQ,B09WFWT9VR,B01J4U20D6,B01N75JV14,B0DB5RVQLB,B075MZLM1K,B06XFY1W6T,B075MZN12T,B0DB5D3QCY,B0DB5RQHFR,B00DLTBV4Q,B0CKSCPX3J,B07QGX3K32,B0GFD35QB7,B06XBLY9D3,B0GFDKQLBS,B0DB5PBR29,B06XBLDM9W,B0FVDT8R1F,B00OOJMY02,B00OOJMUAG,B0DB5RSZNH,B0BY94JD6K,B0D3GSR736,B0FVDWFL5C,B00UH9ADP6,B01BJ6NWGM,B0D3FNYW1Y,B06XBYGT6H,B00UGN90NY,B0DW3Q7X31,B00DU5681W,B06XBKZKSY,B08GPFR7YH,B0G2L4HWW7,B08TBFLM8K,B0DB5QKJFG,B06XC1ZHFN,B0DB5RBXC9,B01M2X5UQN,B0DZ2J2LHK,B01CC8SAXG,B0DB4TTR6Z,B0DZ2JQRST,B0DB5S9P6L,B0FJG3FYB6,B0D55P18ST,B00EN6QSQW,B0DB5SC5L7,B0CNTMPT18,B06XFT3THZ,B0B8CPR62G,B06XBJ9Z2M,B06XBJ9Z2R,B00UGN8SVY,B0CB55F75P</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="17.25" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -8060,6 +8075,11 @@
           <t>중~대형견 대상; センシブル 키워드 포함; 알러지/소화/피부/체중 케어 유사</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>B0763S75ZG,B0763W5KYN,B0BWJ3HYVX,B08TBFLM8K,B07PKM49Z1,B00DU5681W,B0DK8Q7RCB,B0CJHQMSMQ,B09T33GCR3,B06XBKZKSY,B0BY954JJR,B0CJHM5WNP,B01N47EL7T,B0BY92VNKW,B0BY9647B1,B0BY971391,B06XBWFSQ7,B0D3FXM3S4,B00ZHE5XNS,B0CZXN6YD2,B0BXCN1MYL,B0DKNF6GRK,B0F2FCC3ZG,B0GCLLSXVJ,B06XC1WH9C,B085956C14,B0B5743XTQ,B0GCMD8KVZ,B0FNN2MGCT,B09T9PR8P8,B0BZCBB7FS,B09CL2G3YR,B0B8CNCTKV,B07VC6Z5YZ,B00UGN90NY,B0BLGSGRSX,B06XFTN1VK,B0FKGK87YS,B081MPJM31,B07GXJCW4V,B086GNFX5N,B0GCMK97CG,B01J4U1T5G,B00EN6QSIU,B014R2804O,B014QS48GI,B0DLWWGTQV,B00UGN9CK0,B07B2TC59J,B0812FZSW2,B097P5BXJ6,B07Y1S4RMV,B0DK8RQFVS,B075MZLM1K,B075MZN12T,B0G56KGPRV,B01N75JV14,B0FVDT8R1F,B0DWMJ53Z3,B09G652JK9,B00DLTBV4Q,B0FVL5YR5L,B0F3JYKFHG,B0873C3VNJ,B0FVFDFZXG,B0BHHLNYXV,B07QGX3K32,B0DK8S2F7X,B0DZX9778S,B0FJG3FYB6,B0FVDNG4G1,B0DJVDQWDW,B0D3GSR736,B0DQ7ZK222,B08NP6ZHTJ,B08NVT445G,B08NPRG7WF,B0DQ8231CK,B0DQ7YVV4Q,B0DKF7QPS6,B0CPY165M5,B0BHHL9M6B,B08M5F8XD7,B08NP9ZZZ1,B0DK8RHYX6,B0DQ7XFHCZ,B087LR5GY3,B0DN1P332G,B0DN1H8D78,B0DN1Q8S52,B0DN1JTP5L,B0DN1H4BHN,B0DN1KJQQD,B0DN1LDLG9,B0DN1PM7KH,B0DN1PK6XK,B0DN1K5Q55,B0DSZWN97N,B0DN1KCZ43</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -8127,6 +8147,11 @@
           <t>고양이 케어(체중/신장) 키워드 일치</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>B075D1R3D3,B0D1KV2KGB,B08JZJC4SM,B01J4U20MM,B08L376566,B08YR2ZR3H,B08XLQ2G98,B0FBFKPGWS,B0CNTM9YGF,B08YR3379W,B0DK8S86JQ,B00MGL2EJ6,B0CG1KW61F,B0CG1MNP16,B09S3J31SS,B0CG1LHQGD,B01J4U1F0U,B00MFBEYGS,B0D21NMPL4,B0CVS59MYS,B00MFBEO7M,B0GCBWTZ6B,B09SZBVDQY,B0BZGNBQR3,B0CG1NN5W2,B07SJS6KJ1,B0FV7NLSXS,B0F88SYJ37,B08XVHFS5F,B0CG1L1HJS,B01J4U1N7A,B004VCDZ14,B0CNTNDSXJ,B0D1XVJFYV,B0GBGDNCRY,B08514YML7,B0FP48BQ46,B0D1XXVB6N,B0DTJJWZ1B,B07G3T34K8,B007F45NRY,B0D1XYVF3Q,B07G3T7DSF,B0F9PWC456,B0CSFD1HC5,B0DXKKSHFC,B0DTTZMLKX,B0DHZ4KYL7,B0DK8ST7T7,B0DQYPFPSG,B0C3BC31CP,B08KGG1DZT,B0G4CH5YXM,B0G4CCVR65,B0FX41FVXS,B0FX43JVL6,B0DHX2X75G,B0G6JJMBMD,B08514SDJ4,B0G6JK2JGG,B0G4CCMD2C,B0FX41B986,B0DHX5H878,B0G6KC43TP,B0FXFKWNPZ,B0DSHZ5K1F,B0C8MVHCL6,B0DZX97HM7,B01M7TEXAF,B0DSHX4CGP,B07ZVM38GL,B09TQLX49M,B0CVRR9LHH,B07Y1V1NLP,B0BG2DRNV5,B0DX5X81Q8,B09TNL26VG,B00UAQR57A,B00NHGLX8W,B09V2F5SSY,B09S3KY6Z3,B0DCN1LG49,B09TNS86JR,B0DN1MKG37,B0DN1MYJBS,B0DHKQL7CR,B0DN1QM21Y,B0DN1J4JG5,B0DN1JSXYX,B0DN1KT1MD,B0DN1MYJD7,B0DN1MB7SS,B0DN1MRFPR,B079ZRWVW9,B0DHKN8BZK</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -8194,6 +8219,11 @@
           <t>고양이 데ンタル/대립 키워드 유사</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>B0FNMRDZ9G,B0D6S314YT,B0D8KCBW7K,B0BLH89XXQ,B0185JPH3C,B08ZCJP7PB,B0DZ2H184V,B0D7M9ZRXW,B01CZKIVJ4,B09WFR6YRZ,B0DCNBN6Y8,B0BLGNV677,B08CXPX4RZ,B079ZDB5DH,B0D5PMTM8W,B0DJSHNN4B,B09WGHD8P7,B08567967Q,B0857XPWF9,B0DB5THXQK,B0DTYLD5F1,B07FD86BRZ,B0DB5T1B6K,B0FN7PCNTW,B0DHNV9K73,B00WOMHY42,B0F6NPZM1V,B0FCCGGDBX,B0F6LS8JWL,B0F6DGCC36,B0BG48716N,B01GTF9NDO,B0B92LC7ZQ,B006S9FFT8,B0DCSL1QHH,B0F6CXKNRM,B0F513QXFV,B0FT41QG71,B0F6LYD79K,B0F4XSG2JQ,B0F6PKWF7M,B0F4Y151JS,B0F51W3JN1,B0F4XYTXSN,B0F52WRWCD,B0F53LLQZ9,B0F4XTQSJ6,B0F4ZCJHCM,B0DW3WHSTH,B0BJV9HXLJ,B0BVPLQJPT,B07PCXTWD2,B0BVP5MH2K,B0BVPBN3RC,B007F45LIK,B09WMX3CWQ,B0D1XP8VWB,B08W5WV3YG,B0CG1NV6P2,B08YRQCNS1,B0D7M7KRDZ,B0DW3LTX8C,B07RWSYLHW,B075MYRNC1,B08LRFNGTZ,B007F45NRY,B0BVNV4T48,B0BVPW4LKD,B0BVPS9H3N,B0D1Y1ZK2K,B07G37VPH1,B0DCNFWFG1,B085XRPX83,B0CG1LPYQY,B0CVS3565B,B08YRLTHGY,B092MDJKCW,B0028N3EWS,B07PCQ697V,B0DLGXW8FW,B079ZV5JDN,B0CNTM9YGF,B0B9MMPGGH,B0CKSCC7RH,B09WMYVJGH,B0F9T8Y4Z5,B0DWWZJKJX,B007F45LKS,B09SZBVDQY,B0BVNWP2DR,B07H4DM74Z,B0BLGJDRLV,B09MKB8D22,B0BZGVHRWM,B0DYNSZ1LS,B0756XJMVV</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="17.25" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -8244,6 +8274,11 @@
           <t>중~대형견 체중관리(저지방/ライト) 성격 유사</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>B0763S75ZG,B0763W5KYN,B0BWJ3HYVX,B06XFY1W6T,B07PKM4FNK,B01CC8S6BM,B07P354PVN,B06XBJ9Z2R,B00ESB357C,B00ESB379I,B0756YQ6FZ,B01J4U1F78,B08XY4GJH6,B07B4F31JG,B00DLTBV4Q,B07GXGF4RD,B075D1H1YS,B00UR25RFE,B0BQRFKN92,B0CF1QDTHR,B0B8CNZ4M8,B0B8CKM6HN,B00UR25R04,B01CC8SF1S,B0CJLHF4FD,B0CDTDMSMR,B00ESB3522,B01C6UDO0E,B0FCXYYLB8,B01CC8SEXM,B08NP9ZZZ1,B0CQ2NQZPM,B07GXHW63N,B09VGFZD7T,B0BY967V1C,B0D4QQWQ3F,B06XBVNPCC,B09BFCNRTY,B06XBLG2VQ,B01J4U1N5M,B0B8CLB199,B07GXJG4FD,B0DK8S2F7X,B00UR25W4U,B06XBVNMRZ,B00ESB34YQ,B0FCY1ZP3Y,B0CJHM5WNP,B0FNN2MGCT,B01C6R0O82,B0CJHQMSMQ,B0GCM31VL8,B0F5H12V4W,B0CCYK1X2K,B00IN5F838,B0BH3574FW,B079ZPN429,B0BFLCLB14,B083YR28VF,B01C6TDXPG,B081MPJM31,B0BY94GLQ3,B06XBMV58J,B06XC45LHG,B01C6U961K,B01N47EL7T,B00ADX5DGA,B01CC8SAXG,B09BFBK12X,B00M0F8CBW,B09BFBSLWX,B06XFSFQK6,B0851YKBT4,B000WAC1K0,B06XC1WKT4,B09VGS86R7,B01G81TDES,B0BWDRMD9Z,B0BWDSDXDG,B00CIMXIAC,B0FPFTBSMD,B06XC2P7C8,B07VC6Z5YZ,B001PS5TMU,B075MZN12T,B086GNFX5N,B009ZSMU7E,B0GFDB3MTM,B00OYTYYLO,B089GM1C22,B0BBKW4YNF</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="17.25" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -8294,6 +8329,11 @@
           <t>소형견 미니 라인; 시니어/라이트(체중관리) 키워드 유사</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>B00EN6QSIU,B07B4F31JG,B00EN6QVQ4,B01CC8SEXM,B086F3P6G8,B01CC8SEZA,B01CC8SAXG,B01CC8SAM2,B00EN6QSQW,B0BY93SKMQ,B0DD3LQWQH,B01CC8SF54,B06XBLG2VQ,B01K4BGXYQ,B007IE6QO0,B0D3FXM3S4,B09BQ7648X,B08DNNPMGB,B0DZ2JQRST,B0CVS63DHB,B079Z9H36K,B06XFTN1VK,B09VGS86R7,B0CSYMCBJX,B0CX54SVGD,B0B3RJZWRF,B01J4U20OK,B0BCK9RT7R,B01J4U1TDI,B07Z8C3ZFH,B01C6UHTAU,B06XBYGT6H,B01C6R0TRS,B06XC1ZHFN,B07KXTJP4H,B01CC8SF1S,B0D1Y8GYSG,B01LEQVHBE,B09M84SDFN,B075D1H1YS,B06XC3WZJ8,B09BN3BLJ9,B06XBJ9Z2R,B09T8YHF9F,B075D4LTK6,B07Z8C3BHV,B01J4U16W2,B0BWJ3HYVX,B00ESB379I,B0756YQ6FZ,B01J4U1F78,B00ESB357C,B07GXGF4RD,B08XY4GJH6,B0CF1QDTHR,B0CQ2NQZPM,B07GXHW63N,B00ESB3522,B0CCYK1X2K,B0CJ4XBZQZ,B0B8CPB24C,B0CDTDMSMR,B09S3NJQ9B,B0CQ2PRLMB,B06XC2P7C8,B0CK7YNT5K,B0DJVDJ2L5,B0DJVF774X,B0DJVDGRSZ,B0C3QR3Y33,B00ZZB2QKQ,B0FH1YPRL6,B0FH1Y58SF,B0FLVXWN2G,B0FLZ92N37,B0D2YCCBXH,B0FH1Z6NVP,B0FH1ZDBQP,B01J4U1N5M,B0FH1Y73QC,B0FH21M8RP,B0FLVXGCXF,B0FLZT3JR4,B0FP6QYZGZ,B0FH22PNY7,B0FLZPL5BR,B0FLVWZ298,B0FMP8QCPF</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="17.25" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -8378,6 +8418,11 @@
           <t>자견(パピー/ジュニア) 대상; 소화/피부 케어 유사</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>B01CUWLSY2,B005OI7J98,B07GXJ237Y,B07GXHL24Z,B07PKM4FNL,B0D4JXPT8H,B075D1L97V,B00UGN8MCE,B072BB6WQ5,B06XBLC1FM,B0B9MMX8SQ,B0BY941PZL,B06XBTJFGC,B0BBKW4YNF,B00EN6QN9Y,B06XFPYQZ2,B0FV8GJYKN,B0BHHLNYXV,B06XBMQW48,B0BY9583WC,B07Y1S4RMV,B0DK8RQFVS,B075MZLM1K,B075MZN12T,B0G56KGPRV,B01N75JV14,B0FVDT8R1F,B0DWMJ53Z3,B09G652JK9,B00DLTBV4Q,B0FVL5YR5L,B0F3JYKFHG,B0873C3VNJ,B0FVFDFZXG,B07QGX3K32,B0DK8S2F7X,B0DZX9778S,B0FJG3FYB6,B0FVDNG4G1,B0DJVDQWDW,B0D3GSR736,B0DQ7ZK222,B08NP6ZHTJ,B08NVT445G,B08NPRG7WF,B0DQ8231CK,B0DQ7YVV4Q,B0DKF7QPS6,B0CPY165M5,B0BHHL9M6B,B08M5F8XD7,B08NP9ZZZ1,B0DK8RHYX6,B0DQ7XFHCZ,B087LR5GY3,B0DN1P332G,B0DN1H8D78,B0DN1Q8S52,B0DN1JTP5L,B0DN1H4BHN,B0DN1KJQQD,B0DN1LDLG9,B0DN1PM7KH,B0DN1PK6XK,B0DN1K5Q55,B0DSZWN97N,B0DN1KCZ43,B0BZCBB7FS,B09T33GCR3,B0CC42XYKQ,B00DU5681W,B0CC457Z3V,B014R25TCK,B08TBFLM8K,B06XFY8PBC,B0FBW2Y9VY,B06ZZ5JXHG,B09CL32RQB,B09CL2G3YR,B09CL2QTPL,B01M2X5UQN,B09CL39XS5,B0DSZM81RT,B01BYLXT7O,B06Y1VJBNN,B06XFG1823,B06XFY954X,B0DSZVDX86,B06XFSDCPK,B0DSZJHZLJ,B0DSZRFQVF,B0DSZV8T2R,B06XFYXMLH,B0DSZZM6CM,B0DQ7YYGDJ,B09FLHTRM2,B0CC45278W,B0DHKJ14N3,B06XFTVZKX,B06XFSRQ9M,B06XFZFQDG,B06XFX2LY8</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="17.25" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
@@ -8428,6 +8473,11 @@
           <t>VET(처방식) + 비만(肥満/ダイエット) 키워드 일치</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>B0DK8S2F7X,B0DK8RHYX6,B00DLTBV4Q,B07B4F31JG,B0BY967V1C,B07Y1S4RMV,B01M7WPP0N,B075MZN12T,B075MZLM1K,B00DU5681W,B09T33GCR3,B06XBKZKSY,B0F3JYKFHG,B0D3GSR736,B0D1XWZ3KV,B01M7TEXAF,B06XBVNPCC,B079ZPN429,B0BY94GLQ3,B0DHKMGVWF,B0DHKFVVWV,B0DQ7ZK222,B0DHKDPPGM,B0DQ8231CK,B0DHKGBH8B,B075MYRNC1,B0DHKJ14N3,B07Y1V1NLP,B0DHKHR63K,B0DHKQXWZB,B01MAWHCN5,B0011NJOKW,B0D4F1NH1X,B0DHKNXQ53,B0DHKFHQP1,B0DHKHXNWZ,B0DHKPCB9B,B0DHKGGYJ2,B0DHKR6LR8,B0DHKHX3XK,B0DHKQ22PL,B0DHKJQ953,B0DHKJLWL7,B0DHKR9HKZ,B0DHKGN5KY,B0DHKDHY4S,B0DHKGJRVY,B0DHKHZRN9</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="17.25" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -8461,6 +8511,11 @@
           <t>VET(처방식) + 소화기(消化器) 키워드 일치</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>B0DK8RQFVS,B0CSDJ3MQ8,B075MZLM1K,B0CL2QZ1VZ,B07BF7M62D,B0FVDT8R1F,B07Y1S4RMV,B075MZN12T,B0FVDWFL5C,B0FVFDFZXG,B0FVL5YR5L,B0DWMJ53Z3,B0F3JYKFHG,B0FVDVQ6FQ,B00DLTBV4Q,B0G23YT6H6,B0G56KGPRV,B0DK8S2F7X,B0DZX9778S,B01N75JV14,B0D3GSR736,B0FVDNG4G1,B075MYRNC1,B0DK8RHYX6,B0BZCN6QX8,B08NP6ZHTJ,B08NP9ZZZ1,B0DQ7ZK222,B08NVT445G,B08NPRG7WF,B0CPY165M5,B0011NJOKW,B0DQ8231CK,B0DQ7YVV4Q,B087LR5GY3,B0DQ7XFHCZ,B0DN1Q8S52,B0DN1H4BHN,B0DN1P332G,B0DN1H8D78,B0DN1KJQQD,B0DN1JTP5L,B0DN1PK6XK,B0DN1K5Q55,B0DN1PM7KH,B0DN1LDLG9,B0DN1MRZ2M,B0DN1MPS8J</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="17.25" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
@@ -8511,6 +8566,11 @@
           <t>강아지 신장(腎臓) 케어 키워드 유사 (VET 포함/비포함 모두)</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>B0DK8TBG29,B09P5JH4WM,B0DK8SW8FT,B0B8YWV3DT,B0DK8RB5B1,B01M7TEXAF,B0DQ7ZK222,B0DK8RHYX6,B0FVDNG4G1,B0DQ7XFHCZ,B08514SDJ4,B0DN1P332G,B0DHKRBZDZ,B0DHKMGVWF,B0DN1H4BHN,B0DHKGC5WC,B0DHKTFMWP,B0DHKRZYDP,B0DHKR5RV2,B0DHKFT713,B0DHKKZC48,B0DN1LKY6M,B0DN1KJQQD,B0DN1KC49R,B0DHKFVVWV,B0DHKQ22PL,B0DHKR857Y,B0DHKGH54Q,B0DHKHVW3F,B0DHKJGZQQ,B0DK8RKYMH,B08RZDVDYH,B0DHKKCZYW,B0DHKHM1K5,B0DHKT4Y4L,B0DN1PH3L2,B0DHKPRBN9,B0DHKGPSD6,B0DHKR5J9F,B0DHKRN9K6,B0DHKKM9CZ,B0DHKR1SCW,B0DHK9KR3H,B0DHKLYCV8,B0DHKDPPGM,B0DHKD8S95,B0DHKKFDBM,B0DN1P4SW2,B0CV5VN7PJ</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="17.25" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
@@ -8627,6 +8687,11 @@
       <c r="F31" t="inlineStr">
         <is>
           <t>자묘(子猫)/ジュニア 키워드 일치</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>B007F45LKS,B0BJV9HXLJ,B007F45LIK,B085XR6ZXK,B00EN6QG0K,B0B3RHS74H,B09R1LKY4J,B079ZP8KR2,B07G37VPH1,B07G715H52,B071KSN4BD,B0756YJLDH,B09S31JDRJ,B09V2MCQ22,B07G735HWR,B07P64XXPY,B007F45NP6,B08XVDRJDJ,B07PCXTWD2,B09S3KY6Z3,B085XRV2KC,B08R5PG2FD,B08XVDXPXJ,B01N4TBBJD,B0CG1KS19C,B0DW3WHSTH,B07P7GD2TY,B09N724BZ9,B092MDJKCW,B0DYNQVZGL,B0B9MQQTFC,B09V2MLD99,B00MFBEYMM,B0CG1L1HJS,B01N27NVZM,B085XRPX83,B08XLQ2G98,B0DWX5S727,B0BTPQB9H7,B0DXFB5FF5,B0F2SJNPYF,B0B9MMPGGH,B06XPPDZ3X,B01LWNTS4B,B09JFZ6BSL,B0CVS3565B,B0CGX1NMSP,B0DCNFWFG1,B0DCNG3DFK,B0DCNB52VK,B0DYNSVVXQ,B0BZGVHRWM,B0DHGP3WVC,B07GXHQJS4</t>
         </is>
       </c>
     </row>

</xml_diff>